<commit_message>
Add leakage-safe forecasting and meta-learning updates
</commit_message>
<xml_diff>
--- a/artifacts/reports/architecture_tuning_final_shortlist_v1.xlsx
+++ b/artifacts/reports/architecture_tuning_final_shortlist_v1.xlsx
@@ -675,7 +675,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>esn_g004</t>
+          <t>esn_g001</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -685,7 +685,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>esn_grp_004</t>
+          <t>esn_grp_001</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -694,25 +694,25 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0.02708031392595043</v>
+        <v>0.02688398473803453</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0356904542540013</v>
+        <v>0.0354940319068306</v>
       </c>
       <c r="I2" t="n">
-        <v>1.799980602176624</v>
+        <v>1.777841596169583</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5036647406265818</v>
+        <v>0.5124012686382303</v>
       </c>
       <c r="K2" t="n">
-        <v>0.3956744925936046</v>
+        <v>0.3243366101847238</v>
       </c>
       <c r="L2" t="n">
-        <v>0.2448261407359192</v>
+        <v>0.1615128481490602</v>
       </c>
       <c r="M2" t="n">
-        <v>23.05802279986286</v>
+        <v>17.49058050001622</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -739,19 +739,19 @@
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="n">
-        <v>160</v>
+        <v>64</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.92</v>
+        <v>0.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.001</v>
+        <v>0.0001</v>
       </c>
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr"/>
@@ -771,7 +771,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>chaotic_esn_g003</t>
+          <t>chaotic_esn_g002</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>esn_grp_003</t>
+          <t>esn_grp_002</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -790,25 +790,25 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.02820228800932287</v>
+        <v>0.0277351448000609</v>
       </c>
       <c r="H3" t="n">
-        <v>0.037438382422971</v>
+        <v>0.0369656877673297</v>
       </c>
       <c r="I3" t="n">
-        <v>1.882370987521124</v>
+        <v>1.847625638623427</v>
       </c>
       <c r="J3" t="n">
-        <v>0.5049045619139999</v>
+        <v>0.507410137543855</v>
       </c>
       <c r="K3" t="n">
-        <v>0.3386673259298765</v>
+        <v>0.3538351870365322</v>
       </c>
       <c r="L3" t="n">
-        <v>0.2107616611120411</v>
+        <v>0.1770569629630632</v>
       </c>
       <c r="M3" t="n">
-        <v>19.77944353350904</v>
+        <v>19.11211739998544</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -835,19 +835,19 @@
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
       <c r="X3" t="n">
-        <v>128</v>
+        <v>96</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.0005</v>
+        <v>0.0001</v>
       </c>
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
@@ -886,25 +886,25 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0.02709658818015333</v>
+        <v>0.02682418377440117</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0357511100726672</v>
+        <v>0.0354414435197278</v>
       </c>
       <c r="I4" t="n">
-        <v>1.809845599303096</v>
+        <v>1.776576380209354</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5035695704535579</v>
+        <v>0.5141611277520614</v>
       </c>
       <c r="K4" t="n">
-        <v>0.3442249231523385</v>
+        <v>0.4275162277779061</v>
       </c>
       <c r="L4" t="n">
-        <v>0.2154416509319734</v>
+        <v>0.2149457990742155</v>
       </c>
       <c r="M4" t="n">
-        <v>20.14799666703523</v>
+        <v>23.12863296667638</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -982,25 +982,25 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0.0268690852072813</v>
+        <v>0.02655269885146473</v>
       </c>
       <c r="H5" t="n">
-        <v>0.03528007932162653</v>
+        <v>0.03492366694938973</v>
       </c>
       <c r="I5" t="n">
-        <v>1.749178200279071</v>
+        <v>1.730467779815383</v>
       </c>
       <c r="J5" t="n">
-        <v>0.5089475608459146</v>
+        <v>0.5180384394586097</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1333962527774188</v>
+        <v>0.1325629870378987</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0005216111043139667</v>
+        <v>0.0003669740725416</v>
       </c>
       <c r="M5" t="n">
-        <v>4.821043099742383</v>
+        <v>4.785478599975856</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -1074,25 +1074,25 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0.02870808412912347</v>
+        <v>0.0286413774654754</v>
       </c>
       <c r="H6" t="n">
-        <v>0.03706137151935446</v>
+        <v>0.03703021303409697</v>
       </c>
       <c r="I6" t="n">
-        <v>1.958247411014568</v>
+        <v>1.954107204205077</v>
       </c>
       <c r="J6" t="n">
-        <v>0.5190528144585363</v>
+        <v>0.5120630277927463</v>
       </c>
       <c r="K6" t="n">
-        <v>0.1685884916611636</v>
+        <v>0.1636751870367637</v>
       </c>
       <c r="L6" t="n">
-        <v>0.0006375925990545334</v>
+        <v>0.0006340749985408667</v>
       </c>
       <c r="M6" t="n">
-        <v>6.092139033367857</v>
+        <v>5.915133433270967</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -1166,25 +1166,25 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>0.03180258425642687</v>
+        <v>0.03134430164226327</v>
       </c>
       <c r="H7" t="n">
-        <v>0.04014144151396151</v>
+        <v>0.03964451374446123</v>
       </c>
       <c r="I7" t="n">
-        <v>2.359021158360453</v>
+        <v>2.310245750696164</v>
       </c>
       <c r="J7" t="n">
-        <v>0.4942611883646461</v>
+        <v>0.4979596956413343</v>
       </c>
       <c r="K7" t="n">
-        <v>0.4413634305561168</v>
+        <v>0.4538718129619223</v>
       </c>
       <c r="L7" t="n">
-        <v>0.006114757408525867</v>
+        <v>0.006639984258611099</v>
       </c>
       <c r="M7" t="n">
-        <v>16.10921476672714</v>
+        <v>16.57842469993921</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -1268,25 +1268,25 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>0.02616428792103197</v>
+        <v>0.0262398468955799</v>
       </c>
       <c r="H8" t="n">
-        <v>0.03468600839465524</v>
+        <v>0.0348165631005925</v>
       </c>
       <c r="I8" t="n">
-        <v>1.708343244637535</v>
+        <v>1.725998206960399</v>
       </c>
       <c r="J8" t="n">
-        <v>0.5257469268673777</v>
+        <v>0.5222033881904308</v>
       </c>
       <c r="K8" t="n">
-        <v>0.4175126138940902</v>
+        <v>0.411209099999892</v>
       </c>
       <c r="L8" t="n">
-        <v>0.003555387028932733</v>
+        <v>0.003291591666547167</v>
       </c>
       <c r="M8" t="n">
-        <v>15.15844803322883</v>
+        <v>14.92202489999181</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -1347,7 +1347,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>chaotic_lstm_g003</t>
+          <t>chaotic_lstm_g002</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>lstm_grp_003</t>
+          <t>lstm_grp_002</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1366,25 +1366,25 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0.02631610738831523</v>
+        <v>0.0262683407759386</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0348353914992817</v>
+        <v>0.03482177650678744</v>
       </c>
       <c r="I9" t="n">
-        <v>1.71772321853742</v>
+        <v>1.730576619310517</v>
       </c>
       <c r="J9" t="n">
-        <v>0.5180848701473704</v>
+        <v>0.5149568144995397</v>
       </c>
       <c r="K9" t="n">
-        <v>2.382150407408416</v>
+        <v>1.231674241666581</v>
       </c>
       <c r="L9" t="n">
-        <v>0.0153115287108381</v>
+        <v>0.007017510184528768</v>
       </c>
       <c r="M9" t="n">
-        <v>86.30862970029314</v>
+        <v>44.59290306663994</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -1417,10 +1417,10 @@
         <v>64</v>
       </c>
       <c r="V9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
@@ -1491,12 +1491,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>esn_g004</t>
+          <t>esn_g001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>chaotic_esn_g003</t>
+          <t>chaotic_esn_g002</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1511,12 +1511,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Средний runtime shortlisted-кандидатов: 21.00 sec.</t>
+          <t>Средний runtime shortlisted-кандидатов: 19.91 sec.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Delta MAE (chaotic - practical): 0.0006; хаотические кандидаты сохранены как исследовательский контур.</t>
+          <t>Delta MAE (chaotic - practical): 0.0004; хаотические кандидаты сохранены как исследовательский контур.</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Средний runtime shortlisted-кандидатов: 5.46 sec.</t>
+          <t>Средний runtime shortlisted-кандидатов: 5.35 sec.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Delta MAE (chaotic - practical): 0.0018; хаотические кандидаты сохранены как исследовательский контур.</t>
+          <t>Delta MAE (chaotic - practical): 0.0021; хаотические кандидаты сохранены как исследовательский контур.</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Средний runtime shortlisted-кандидатов: 16.11 sec.</t>
+          <t>Средний runtime shortlisted-кандидатов: 16.58 sec.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>chaotic_lstm_g003</t>
+          <t>chaotic_lstm_g002</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -1606,12 +1606,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Средний runtime shortlisted-кандидатов: 50.73 sec.</t>
+          <t>Средний runtime shortlisted-кандидатов: 29.76 sec.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Delta MAE (chaotic - practical): 0.0002; хаотические кандидаты сохранены как исследовательский контур.</t>
+          <t>Delta MAE (chaotic - practical): 0.0000; хаотические кандидаты сохранены как исследовательский контур.</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>esn_g004</t>
+          <t>esn_g001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1728,19 +1728,19 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>160</v>
+        <v>64</v>
       </c>
       <c r="I2" t="n">
-        <v>0.92</v>
+        <v>0.9</v>
       </c>
       <c r="J2" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="K2" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>0.001</v>
+        <v>0.0001</v>
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -1750,7 +1750,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>chaotic_esn_g003</t>
+          <t>chaotic_esn_g002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1764,19 +1764,19 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>128</v>
+        <v>96</v>
       </c>
       <c r="I3" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="J3" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="K3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0005</v>
+        <v>0.0001</v>
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -1966,7 +1966,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>chaotic_lstm_g003</t>
+          <t>chaotic_lstm_g002</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1986,10 +1986,10 @@
         <v>64</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>architecture_tuning_final_shortlist_v1_20260329T180423Z</t>
+          <t>architecture_tuning_final_shortlist_v1_20260819T080135Z</t>
         </is>
       </c>
     </row>

</xml_diff>